<commit_message>
Unifica sinal de desconto e limpa cabeçalho duplicado do mapa
- OC: Total = Subtotal - Desconto + IPI + Frete + Outros + ICMS, igual
  à convenção do Mapa (antes era tudo soma; desconto só funcionava se
  digitado negativo).
- Mapa: cabeçalho tinha Data e Obra duplicados (B8/C8 x E6/F6, B9/C9 x
  E8:G9) e o campo C.C. sem célula de valor própria (a célula ao lado,
  F7, tinha o texto solto "Obra: " em vez de ficar em branco). Remove
  os campos duplicados e libera F7 como entrada de valor do C.C.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FxrRoRLoVG2FM9fbtbGDds
</commit_message>
<xml_diff>
--- a/templates/mapa_cotacao_modelo.xlsx
+++ b/templates/mapa_cotacao_modelo.xlsx
@@ -3500,16 +3500,8 @@
         </is>
       </c>
       <c r="D6" s="285" t="n"/>
-      <c r="E6" s="384" t="inlineStr">
-        <is>
-          <t>Data:</t>
-        </is>
-      </c>
-      <c r="F6" s="386" t="inlineStr">
-        <is>
-          <t>[DATA]</t>
-        </is>
-      </c>
+      <c r="E6" s="384" t="n"/>
+      <c r="F6" s="386" t="n"/>
       <c r="G6" s="386" t="inlineStr">
         <is>
           <t>Comprador:</t>
@@ -3562,11 +3554,7 @@
           <t>C.C.:</t>
         </is>
       </c>
-      <c r="F7" s="393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Obra: </t>
-        </is>
-      </c>
+      <c r="F7" s="393" t="n"/>
       <c r="G7" s="298" t="n"/>
       <c r="H7" s="395" t="inlineStr">
         <is>
@@ -3598,13 +3586,7 @@
         </is>
       </c>
       <c r="D8" s="285" t="n"/>
-      <c r="E8" s="401" t="inlineStr">
-        <is>
-          <t>[Nome da Obra]</t>
-        </is>
-      </c>
-      <c r="F8" s="303" t="n"/>
-      <c r="G8" s="304" t="n"/>
+      <c r="E8" s="401" t="n"/>
       <c r="H8" s="495" t="inlineStr">
         <is>
           <t>Bruno Felizardo</t>
@@ -3635,9 +3617,6 @@
         </is>
       </c>
       <c r="D9" s="288" t="n"/>
-      <c r="E9" s="307" t="n"/>
-      <c r="F9" s="308" t="n"/>
-      <c r="G9" s="309" t="n"/>
       <c r="H9" s="412" t="n"/>
       <c r="I9" s="413" t="inlineStr">
         <is>
@@ -4333,7 +4312,7 @@
     <filterColumn colId="6" hiddenButton="0" showButton="0"/>
     <filterColumn colId="7" hiddenButton="0" showButton="0"/>
   </autoFilter>
-  <mergeCells count="72">
+  <mergeCells count="71">
     <mergeCell ref="N26:O26"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="L7:M7"/>
@@ -4356,7 +4335,6 @@
     <mergeCell ref="C16:G16"/>
     <mergeCell ref="L24:M24"/>
     <mergeCell ref="N28:O33"/>
-    <mergeCell ref="E8:G9"/>
     <mergeCell ref="N27:O27"/>
     <mergeCell ref="L5:M5"/>
     <mergeCell ref="J27:K27"/>

</xml_diff>

<commit_message>
Fecha buracos de borda no mapa e some com a coluna/linha em branco
- Bordas faltando: canto esquerdo da linha de cabeçalho dos itens, canto
  direito da linha de Subtotal, e as colunas Quant./Unid. inteiramente
  sem borda nas linhas 16-21 (só as linhas 12-15 tinham).
- Coluna A (decorativa, só um "Item orçado" solto) e a linha 1 (vazia)
  ficam com largura/altura quase zero e ocultas, em vez de apagadas:
  ws.delete_rows/delete_cols corrompeu fórmulas (referências não
  ajustadas, viravam auto-referência circular) e chegou a apagar
  valores em colunas com célula mesclada quando testado neste arquivo.
  Resultado visual é o mesmo; nenhuma fórmula foi tocada.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FxrRoRLoVG2FM9fbtbGDds
</commit_message>
<xml_diff>
--- a/templates/mapa_cotacao_modelo.xlsx
+++ b/templates/mapa_cotacao_modelo.xlsx
@@ -494,7 +494,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="64">
+  <borders count="67">
     <border>
       <left/>
       <right/>
@@ -1276,6 +1276,42 @@
         <color indexed="64"/>
       </bottom>
       <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="11">
@@ -1291,7 +1327,7 @@
     <xf numFmtId="164" fontId="22" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="506">
+  <cellXfs count="510">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
@@ -2950,6 +2986,14 @@
     <xf numFmtId="166" fontId="41" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="64" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3352,7 +3396,7 @@
   <dimension ref="A1:P36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="21"/>
   <cols>
-    <col width="3" customWidth="1" style="2" min="1" max="1"/>
+    <col hidden="1" width="0.5" customWidth="1" style="2" min="1" max="1"/>
     <col width="20.28515625" bestFit="1" customWidth="1" style="2" min="2" max="2"/>
     <col width="8.42578125" customWidth="1" style="2" min="3" max="3"/>
     <col width="14" customWidth="1" style="2" min="4" max="4"/>
@@ -3366,7 +3410,7 @@
     <col width="9.140625" customWidth="1" style="2" min="17" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21.75" customHeight="1" thickBot="1">
+    <row r="1" hidden="1" ht="1" customHeight="1" thickBot="1">
       <c r="A1" s="358" t="n"/>
       <c r="B1" s="359" t="n"/>
       <c r="C1" s="359" t="n"/>
@@ -3485,7 +3529,7 @@
           <t>Cotação 03</t>
         </is>
       </c>
-      <c r="O5" s="294" t="n"/>
+      <c r="O5" s="506" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="358" t="n"/>
@@ -3652,12 +3696,8 @@
       <c r="O10" s="312" t="n"/>
     </row>
     <row r="11" customFormat="1" s="19" thickBot="1">
-      <c r="A11" s="422" t="inlineStr">
-        <is>
-          <t>Item orçado</t>
-        </is>
-      </c>
-      <c r="B11" s="423" t="inlineStr">
+      <c r="A11" s="422" t="n"/>
+      <c r="B11" s="507" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
@@ -3824,8 +3864,8 @@
       <c r="E16" s="318" t="n"/>
       <c r="F16" s="318" t="n"/>
       <c r="G16" s="298" t="n"/>
-      <c r="H16" s="499" t="n"/>
-      <c r="I16" s="358" t="n"/>
+      <c r="H16" s="433" t="n"/>
+      <c r="I16" s="398" t="n"/>
       <c r="J16" s="445" t="n"/>
       <c r="K16" s="500">
         <f>H16*J16</f>
@@ -3850,8 +3890,8 @@
       <c r="E17" s="318" t="n"/>
       <c r="F17" s="318" t="n"/>
       <c r="G17" s="298" t="n"/>
-      <c r="H17" s="499" t="n"/>
-      <c r="I17" s="358" t="n"/>
+      <c r="H17" s="433" t="n"/>
+      <c r="I17" s="398" t="n"/>
       <c r="J17" s="445" t="n"/>
       <c r="K17" s="500">
         <f>H17*J17</f>
@@ -3876,8 +3916,8 @@
       <c r="E18" s="318" t="n"/>
       <c r="F18" s="318" t="n"/>
       <c r="G18" s="298" t="n"/>
-      <c r="H18" s="499" t="n"/>
-      <c r="I18" s="358" t="n"/>
+      <c r="H18" s="433" t="n"/>
+      <c r="I18" s="398" t="n"/>
       <c r="J18" s="445" t="n"/>
       <c r="K18" s="500">
         <f>H18*J18</f>
@@ -3902,8 +3942,8 @@
       <c r="E19" s="318" t="n"/>
       <c r="F19" s="318" t="n"/>
       <c r="G19" s="298" t="n"/>
-      <c r="H19" s="499" t="n"/>
-      <c r="I19" s="358" t="n"/>
+      <c r="H19" s="433" t="n"/>
+      <c r="I19" s="398" t="n"/>
       <c r="J19" s="445" t="n"/>
       <c r="K19" s="500">
         <f>H19*J19</f>
@@ -3928,8 +3968,8 @@
       <c r="E20" s="318" t="n"/>
       <c r="F20" s="318" t="n"/>
       <c r="G20" s="298" t="n"/>
-      <c r="H20" s="499" t="n"/>
-      <c r="I20" s="358" t="n"/>
+      <c r="H20" s="433" t="n"/>
+      <c r="I20" s="398" t="n"/>
       <c r="J20" s="445" t="n"/>
       <c r="K20" s="500">
         <f>H20*J20</f>
@@ -3954,8 +3994,8 @@
       <c r="E21" s="318" t="n"/>
       <c r="F21" s="318" t="n"/>
       <c r="G21" s="298" t="n"/>
-      <c r="H21" s="499" t="n"/>
-      <c r="I21" s="358" t="n"/>
+      <c r="H21" s="433" t="n"/>
+      <c r="I21" s="398" t="n"/>
       <c r="J21" s="458" t="n"/>
       <c r="K21" s="505">
         <f>H21*J21</f>
@@ -4000,7 +4040,7 @@
         <f>SUM(O12:O21)</f>
         <v/>
       </c>
-      <c r="O22" s="341" t="n"/>
+      <c r="O22" s="508" t="n"/>
     </row>
     <row r="23" ht="30" customFormat="1" customHeight="1" s="50">
       <c r="A23" s="460" t="n"/>
@@ -4134,7 +4174,7 @@
           <t>Vide observações abaixo.</t>
         </is>
       </c>
-      <c r="O27" s="298" t="n"/>
+      <c r="O27" s="509" t="n"/>
     </row>
     <row r="28" ht="19.9" customFormat="1" customHeight="1" s="33">
       <c r="A28" s="477" t="n"/>

</xml_diff>

<commit_message>
Restaura campo de endereço da obra e fecha a faixa FORNECEDORES
- E6/F6 (Data), F7 (Obra) e o bloco E8:G9 tinham sido removidos por engano
  no commit anterior — não eram duplicata do nome da obra (B9/C9), e sim o
  ENDEREÇO da obra, campo distinto. O rótulo original "[Nome da Obra]"
  nessa célula é que estava errado (deveria dizer "[Endereço completo da
  Obra]"); confirmado com o mapa real que o Bruno usa.
- A faixa "FORNECEDORES" (linha 4) só mesclava até a coluna M, deixando as
  duas células do Fornecedor 3 (N4:O4) soltas, sem a faixa por cima. Agora
  I4:O4 é uma mescla só, cobrindo os três fornecedores.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FxrRoRLoVG2FM9fbtbGDds
</commit_message>
<xml_diff>
--- a/templates/mapa_cotacao_modelo.xlsx
+++ b/templates/mapa_cotacao_modelo.xlsx
@@ -1327,7 +1327,7 @@
     <xf numFmtId="164" fontId="22" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="510">
+  <cellXfs count="511">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
@@ -2994,6 +2994,10 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="44" fillId="2" borderId="10" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3482,7 +3486,7 @@
       <c r="F4" s="291" t="n"/>
       <c r="G4" s="291" t="n"/>
       <c r="H4" s="292" t="n"/>
-      <c r="I4" s="375" t="inlineStr">
+      <c r="I4" s="510" t="inlineStr">
         <is>
           <t>FORNECEDORES</t>
         </is>
@@ -3491,8 +3495,8 @@
       <c r="K4" s="287" t="n"/>
       <c r="L4" s="287" t="n"/>
       <c r="M4" s="287" t="n"/>
-      <c r="N4" s="376" t="n"/>
-      <c r="O4" s="377" t="n"/>
+      <c r="N4" s="287" t="n"/>
+      <c r="O4" s="288" t="n"/>
     </row>
     <row r="5" ht="21.75" customHeight="1" thickBot="1">
       <c r="A5" s="358" t="n"/>
@@ -3529,7 +3533,7 @@
           <t>Cotação 03</t>
         </is>
       </c>
-      <c r="O5" s="506" t="n"/>
+      <c r="O5" s="294" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="358" t="n"/>
@@ -3544,8 +3548,16 @@
         </is>
       </c>
       <c r="D6" s="285" t="n"/>
-      <c r="E6" s="384" t="n"/>
-      <c r="F6" s="386" t="n"/>
+      <c r="E6" s="384" t="inlineStr">
+        <is>
+          <t>Data:</t>
+        </is>
+      </c>
+      <c r="F6" s="386" t="inlineStr">
+        <is>
+          <t>[DATA]</t>
+        </is>
+      </c>
       <c r="G6" s="386" t="inlineStr">
         <is>
           <t>Comprador:</t>
@@ -3598,7 +3610,11 @@
           <t>C.C.:</t>
         </is>
       </c>
-      <c r="F7" s="393" t="n"/>
+      <c r="F7" s="393" t="inlineStr">
+        <is>
+          <t>Obra:</t>
+        </is>
+      </c>
       <c r="G7" s="298" t="n"/>
       <c r="H7" s="395" t="inlineStr">
         <is>
@@ -3630,7 +3646,13 @@
         </is>
       </c>
       <c r="D8" s="285" t="n"/>
-      <c r="E8" s="401" t="n"/>
+      <c r="E8" s="401" t="inlineStr">
+        <is>
+          <t>[Endereço completo da Obra]</t>
+        </is>
+      </c>
+      <c r="F8" s="303" t="n"/>
+      <c r="G8" s="304" t="n"/>
       <c r="H8" s="495" t="inlineStr">
         <is>
           <t>Bruno Felizardo</t>
@@ -3661,6 +3683,9 @@
         </is>
       </c>
       <c r="D9" s="288" t="n"/>
+      <c r="E9" s="307" t="n"/>
+      <c r="F9" s="308" t="n"/>
+      <c r="G9" s="309" t="n"/>
       <c r="H9" s="412" t="n"/>
       <c r="I9" s="413" t="inlineStr">
         <is>
@@ -4036,11 +4061,11 @@
         <v/>
       </c>
       <c r="M22" s="341" t="n"/>
-      <c r="N22" s="464">
+      <c r="N22" s="465">
         <f>SUM(O12:O21)</f>
         <v/>
       </c>
-      <c r="O22" s="508" t="n"/>
+      <c r="O22" s="342" t="n"/>
     </row>
     <row r="23" ht="30" customFormat="1" customHeight="1" s="50">
       <c r="A23" s="460" t="n"/>
@@ -4174,7 +4199,7 @@
           <t>Vide observações abaixo.</t>
         </is>
       </c>
-      <c r="O27" s="509" t="n"/>
+      <c r="O27" s="298" t="n"/>
     </row>
     <row r="28" ht="19.9" customFormat="1" customHeight="1" s="33">
       <c r="A28" s="477" t="n"/>
@@ -4352,7 +4377,7 @@
     <filterColumn colId="6" hiddenButton="0" showButton="0"/>
     <filterColumn colId="7" hiddenButton="0" showButton="0"/>
   </autoFilter>
-  <mergeCells count="71">
+  <mergeCells count="72">
     <mergeCell ref="N26:O26"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="L7:M7"/>
@@ -4363,6 +4388,7 @@
     <mergeCell ref="J10:K10"/>
     <mergeCell ref="N25:O25"/>
     <mergeCell ref="B22:I22"/>
+    <mergeCell ref="I4:O4"/>
     <mergeCell ref="C14:G14"/>
     <mergeCell ref="B27:I27"/>
     <mergeCell ref="E32:H32"/>
@@ -4375,6 +4401,7 @@
     <mergeCell ref="C16:G16"/>
     <mergeCell ref="L24:M24"/>
     <mergeCell ref="N28:O33"/>
+    <mergeCell ref="E8:G9"/>
     <mergeCell ref="N27:O27"/>
     <mergeCell ref="L5:M5"/>
     <mergeCell ref="J27:K27"/>
@@ -4406,7 +4433,6 @@
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="C17:G17"/>
-    <mergeCell ref="I4:M4"/>
     <mergeCell ref="N9:O9"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E31:H31"/>

</xml_diff>